<commit_message>
PolicyTests and CustomerTests added
</commit_message>
<xml_diff>
--- a/src/test/resources/test-data/BookingData.xlsx
+++ b/src/test/resources/test-data/BookingData.xlsx
@@ -4,21 +4,21 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1125" windowWidth="15645" windowHeight="6930" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="1125" windowWidth="15375" windowHeight="7935" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
     <sheet name="login_data" sheetId="4" r:id="rId4"/>
+    <sheet name="customer_profile_data" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:P21"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="71">
   <si>
     <t>First Name</t>
   </si>
@@ -140,14 +140,104 @@
     <t>vikram</t>
   </si>
   <si>
-    <t>vikram1234</t>
+    <t>testName</t>
+  </si>
+  <si>
+    <t>firstName</t>
+  </si>
+  <si>
+    <t>lastName</t>
+  </si>
+  <si>
+    <t>dateOfBirth</t>
+  </si>
+  <si>
+    <t>gender</t>
+  </si>
+  <si>
+    <t>aadhaarNumber</t>
+  </si>
+  <si>
+    <t>panNumber</t>
+  </si>
+  <si>
+    <t>bloodGroup</t>
+  </si>
+  <si>
+    <t>maritalStatus</t>
+  </si>
+  <si>
+    <t>occupation</t>
+  </si>
+  <si>
+    <t>annualIncome</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>pincode</t>
+  </si>
+  <si>
+    <t>updateCustomerProfileTest</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Doctor</t>
+  </si>
+  <si>
+    <t>MG Road</t>
+  </si>
+  <si>
+    <t>Bengaluru</t>
+  </si>
+  <si>
+    <t>Karnataka</t>
+  </si>
+  <si>
+    <t>India</t>
+  </si>
+  <si>
+    <t>vikram123</t>
+  </si>
+  <si>
+    <t>MALE</t>
+  </si>
+  <si>
+    <t>SINGLE</t>
+  </si>
+  <si>
+    <t>ABCDE1234F</t>
+  </si>
+  <si>
+    <t>B_POSITIVE</t>
+  </si>
+  <si>
+    <t>123456789987</t>
+  </si>
+  <si>
+    <t>5000000.00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,6 +257,20 @@
       <name val="Courier New"/>
       <family val="3"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1EB540"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -185,10 +289,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
@@ -199,8 +304,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="1" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -875,7 +983,125 @@
         <v>39</v>
       </c>
       <c r="B2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:P2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
         <v>40</v>
+      </c>
+      <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" t="s">
+        <v>46</v>
+      </c>
+      <c r="H1" t="s">
+        <v>47</v>
+      </c>
+      <c r="I1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" t="s">
+        <v>49</v>
+      </c>
+      <c r="K1" t="s">
+        <v>50</v>
+      </c>
+      <c r="L1" t="s">
+        <v>51</v>
+      </c>
+      <c r="M1" t="s">
+        <v>52</v>
+      </c>
+      <c r="N1" t="s">
+        <v>53</v>
+      </c>
+      <c r="O1" t="s">
+        <v>54</v>
+      </c>
+      <c r="P1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C2" t="s">
+        <v>58</v>
+      </c>
+      <c r="D2" s="9">
+        <v>36809</v>
+      </c>
+      <c r="E2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="G2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H2" t="s">
+        <v>68</v>
+      </c>
+      <c r="I2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" t="s">
+        <v>59</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="L2" t="s">
+        <v>60</v>
+      </c>
+      <c r="M2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N2" t="s">
+        <v>62</v>
+      </c>
+      <c r="O2" t="s">
+        <v>63</v>
+      </c>
+      <c r="P2">
+        <v>554321</v>
       </c>
     </row>
   </sheetData>

</xml_diff>